<commit_message>
Organiza estrutura de extracao, cria painel municipal anual e adiciona data loaders
</commit_message>
<xml_diff>
--- a/dados/info_delegacias/dados_deams_24h.xlsx
+++ b/dados/info_delegacias/dados_deams_24h.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -972,6 +972,125 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Itabaiana</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Lagarto</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Aracaju</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sorocaba</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Palmas</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ariquemes</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>